<commit_message>
correction bouton mMaJ de donnees 4
</commit_message>
<xml_diff>
--- a/matieres.xlsx
+++ b/matieres.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,7 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>categorie</t>
+          <t>cat</t>
         </is>
       </c>
     </row>
@@ -449,16 +449,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MAT101</t>
+          <t>INF101</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mathématiques</t>
+          <t>Algorithmique</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -472,16 +472,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FRA201</t>
+          <t>INF201</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Français</t>
+          <t>Base de données</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -495,20 +495,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HIS301</t>
+          <t>INF301</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Histoire-Géo</t>
+          <t>Programmation Web</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Éveil/Option</t>
+          <t>Fondamentale</t>
         </is>
       </c>
     </row>
@@ -518,20 +518,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SVT401</t>
+          <t>MTH101</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SVT</t>
+          <t>Mathématiques I</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Éveil/Option</t>
+          <t>Fondamentale</t>
         </is>
       </c>
     </row>
@@ -541,20 +541,135 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ANG501</t>
+          <t>MTH201</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Anglais</t>
+          <t>Statistiques</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Éveil/Option</t>
+          <t>Fondamentale</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UO101</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Anglais Technique</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Transversale</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UO102</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Transversale</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RT101</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Réseaux Locaux</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Fondamentale</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GC101</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Résistance des Matériaux</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Fondamentale</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GL401</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Génie Logiciel Avancé</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fondamentale</t>
         </is>
       </c>
     </row>

</xml_diff>